<commit_message>
end of sprint 3/ final sprint artifacts docs
</commit_message>
<xml_diff>
--- a/Documents/Project 3 Requirements.xlsx
+++ b/Documents/Project 3 Requirements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riley\Desktop\dododojo\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19132\Documents\GitHub\project3\dododojo\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3211B167-08B4-4DF6-A95A-4368F384FFC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{311B3CFD-7DE0-4F19-8BA7-7B0C5582A184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{3114261F-E3D0-496D-89B9-05D096F1C2E1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3114261F-E3D0-496D-89B9-05D096F1C2E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Reference Stories" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="94">
   <si>
     <t>Reference Story No.</t>
   </si>
@@ -291,9 +291,6 @@
     <t>Dustin</t>
   </si>
   <si>
-    <t>Create endpoint to send all possible the cards to the front end</t>
-  </si>
-  <si>
     <t>Display the character information and information about their current deck and cards in their possession</t>
   </si>
   <si>
@@ -312,14 +309,23 @@
     <t>create diagram about each card type and its advantages</t>
   </si>
   <si>
-    <t>Users are able to delete their account and all account information</t>
+    <t>added a delete button to the gameplay homescreen to delete account</t>
+  </si>
+  <si>
+    <t>create random encounter for any sprite elements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Final Sprint </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,15 +732,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D145CAD5-F858-4BC1-9902-44B98103FB35}">
   <dimension ref="A1:D26"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="89.125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="89.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -748,7 +754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28.5">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -762,7 +768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.5">
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -776,7 +782,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.5">
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -790,7 +796,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.5">
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -804,7 +810,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="42.75">
+    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -818,7 +824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.5">
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -832,7 +838,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="42.75">
+    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -846,7 +852,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="42.75">
+    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -860,7 +866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="42.75">
+    <row r="10" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -874,7 +880,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36.6" customHeight="1">
+    <row r="11" spans="1:4" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -888,7 +894,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="2" customFormat="1" ht="46.35" customHeight="1">
+    <row r="12" spans="1:4" s="2" customFormat="1" ht="46.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -902,7 +908,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="42.75">
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -916,7 +922,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="42.75">
+    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -930,7 +936,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="42.75">
+    <row r="15" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -944,7 +950,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="69.75" customHeight="1">
+    <row r="16" spans="1:4" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -958,7 +964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="28.5">
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -972,7 +978,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="59.25" customHeight="1">
+    <row r="18" spans="1:4" ht="59.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -986,7 +992,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="67.5" customHeight="1">
+    <row r="19" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1000,7 +1006,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="42.75">
+    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1014,7 +1020,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="42.75">
+    <row r="21" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1028,7 +1034,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="29.25" customHeight="1">
+    <row r="22" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1042,7 +1048,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="28.5">
+    <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1056,7 +1062,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="42.75">
+    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1070,7 +1076,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="57">
+    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1084,7 +1090,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="42.75">
+    <row r="26" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1106,16 +1112,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{562A978C-3608-4AB8-BC01-F8ABFDE138F4}">
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.125" customWidth="1"/>
-    <col min="2" max="2" width="65.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" customWidth="1"/>
+    <col min="2" max="2" width="65.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
@@ -1135,7 +1141,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1155,7 +1161,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1168,11 +1174,14 @@
       <c r="D3">
         <v>1</v>
       </c>
+      <c r="E3" t="s">
+        <v>92</v>
+      </c>
       <c r="F3" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1192,7 +1201,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28.5">
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1212,7 +1221,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1232,7 +1241,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="45">
+    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1252,7 +1261,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1272,7 +1281,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1292,7 +1301,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1312,7 +1321,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.5">
+    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1325,11 +1334,14 @@
       <c r="D11">
         <v>1</v>
       </c>
+      <c r="E11" t="s">
+        <v>92</v>
+      </c>
       <c r="F11" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="28.5">
+    <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1342,11 +1354,14 @@
       <c r="D12">
         <v>1</v>
       </c>
+      <c r="E12" t="s">
+        <v>92</v>
+      </c>
       <c r="F12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="28.5">
+    <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1359,11 +1374,14 @@
       <c r="D13">
         <v>1</v>
       </c>
+      <c r="E13" t="s">
+        <v>92</v>
+      </c>
       <c r="F13" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1383,7 +1401,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="28.5">
+    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1403,7 +1421,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1423,7 +1441,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1443,7 +1461,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1463,7 +1481,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1483,7 +1501,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1496,11 +1514,14 @@
       <c r="D20">
         <v>2</v>
       </c>
+      <c r="E20" t="s">
+        <v>92</v>
+      </c>
       <c r="F20" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="28.5">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1513,11 +1534,14 @@
       <c r="D21">
         <v>2</v>
       </c>
+      <c r="E21" t="s">
+        <v>80</v>
+      </c>
       <c r="F21" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1537,7 +1561,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1557,7 +1581,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="28.5">
+    <row r="24" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1570,16 +1594,19 @@
       <c r="D24">
         <v>2</v>
       </c>
+      <c r="E24" t="s">
+        <v>93</v>
+      </c>
       <c r="F24" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -1594,7 +1621,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1602,50 +1629,59 @@
         <v>84</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="28.5">
+        <v>3</v>
+      </c>
+      <c r="E26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="5" t="s">
         <v>85</v>
       </c>
       <c r="C27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D27">
         <v>3</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="F27" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="28.5">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>86</v>
+      <c r="B28" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="C28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28">
         <v>3</v>
       </c>
+      <c r="E28" t="s">
+        <v>60</v>
+      </c>
       <c r="F28" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="28.5">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1653,10 +1689,10 @@
         <v>88</v>
       </c>
       <c r="C29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>60</v>
@@ -1665,27 +1701,27 @@
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E30" t="s">
         <v>60</v>
       </c>
       <c r="F30" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1699,7 +1735,7 @@
         <v>3</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F31" t="s">
         <v>83</v>
@@ -1707,7 +1743,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1939,20 +1974,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="90df4e60-c7e0-48c4-9d2f-0b08e3213e73" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="90df4e60-c7e0-48c4-9d2f-0b08e3213e73" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1975,26 +2010,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06F02AC8-94BB-4B29-9EB3-1C3BE08341BC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="29236149-13bb-43d3-8a26-87399c13efb2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="90df4e60-c7e0-48c4-9d2f-0b08e3213e73"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A498016-2968-4386-81CE-86C8D27A70AB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06F02AC8-94BB-4B29-9EB3-1C3BE08341BC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="90df4e60-c7e0-48c4-9d2f-0b08e3213e73"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="29236149-13bb-43d3-8a26-87399c13efb2"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>